<commit_message>
Phase 0: Leakage & Metadata Sterilization (R-001..R-004, F-033, F-036, F-039)
Sterilize Public xlsx for DD-grade investor distribution:
- Remove 7 "Internal" leakage occurrences (F-001/002/009/010/011), preserve IRR term
- Strip absPath from workbook.xml (F-003)
- Clean core.xml: Author→TrendStudio, clear description/keywords L3 (F-020/021/022)
- Fix dangling '=' in 17_Deal_Structures B31 (F-036)
- Remove computer:// reference from changelog (bonus)
- Delete 35 backup/bak/FUSE/lock files from Investor_Package (F-039)
- Fix verify.py hardcoded 14 → len(INPUT_FILES) (F-033/R-024)
- Add pipeline/sterilize.py with verify_sterilization()
- Add 34 new Phase 0 tests (test_30_sterilize.py)
- Full suite: 357 passed, 5 skipped, 0 failed (was 323)

https://claude.ai/code/session_01VBjjAoPwBenTgnAprubLW7
</commit_message>
<xml_diff>
--- a/investor_model_v1.0_Public.xlsx
+++ b/investor_model_v1.0_Public.xlsx
@@ -6385,52 +6385,52 @@
           <t>Cash (Денежные средства) &amp; equivalents</t>
         </is>
       </c>
-      <c r="D7" s="729">
+      <c r="D7" s="729" t="n">
         <v>343.95</v>
       </c>
-      <c r="E7" s="729">
+      <c r="E7" s="729" t="n">
         <v>219.02</v>
       </c>
-      <c r="F7" s="729">
-        <v>74.71</v>
-      </c>
-      <c r="G7" s="729">
+      <c r="F7" s="729" t="n">
+        <v>74.70999999999999</v>
+      </c>
+      <c r="G7" s="729" t="n">
         <v>713</v>
       </c>
-      <c r="H7" s="729">
+      <c r="H7" s="729" t="n">
         <v>724.3</v>
       </c>
-      <c r="I7" s="729">
+      <c r="I7" s="729" t="n">
         <v>1071.67</v>
       </c>
-      <c r="J7" s="729">
+      <c r="J7" s="729" t="n">
         <v>1852.59</v>
       </c>
-      <c r="K7" s="729">
+      <c r="K7" s="729" t="n">
         <v>2005.12</v>
       </c>
-      <c r="L7" s="729">
+      <c r="L7" s="729" t="n">
         <v>2189.75</v>
       </c>
-      <c r="M7" s="729">
+      <c r="M7" s="729" t="n">
         <v>2858.6</v>
       </c>
-      <c r="N7" s="729">
+      <c r="N7" s="729" t="n">
         <v>3360.26</v>
       </c>
-      <c r="O7" s="729">
+      <c r="O7" s="729" t="n">
         <v>3546.61</v>
       </c>
-      <c r="P7" s="729">
+      <c r="P7" s="729" t="n">
         <v>2549.52</v>
       </c>
-      <c r="Q7" s="729">
+      <c r="Q7" s="729" t="n">
         <v>1778.29</v>
       </c>
-      <c r="R7" s="729">
+      <c r="R7" s="729" t="n">
         <v>1223.89</v>
       </c>
-      <c r="S7" s="729">
+      <c r="S7" s="729" t="n">
         <v>891.75</v>
       </c>
       <c r="T7" s="514" t="inlineStr">
@@ -6580,52 +6580,52 @@
           <t>ИТОГО АКТИВЫ (АКТИВЫ) (ИТОГО АКТИВЫ)</t>
         </is>
       </c>
-      <c r="D10" s="726">
+      <c r="D10" s="726" t="n">
         <v>424.03</v>
       </c>
-      <c r="E10" s="726">
+      <c r="E10" s="726" t="n">
         <v>399.18</v>
       </c>
-      <c r="F10" s="726">
+      <c r="F10" s="726" t="n">
         <v>374.95</v>
       </c>
-      <c r="G10" s="726">
+      <c r="G10" s="726" t="n">
         <v>987.14</v>
       </c>
-      <c r="H10" s="726">
+      <c r="H10" s="726" t="n">
         <v>1076.76</v>
       </c>
-      <c r="I10" s="726">
+      <c r="I10" s="726" t="n">
         <v>1359.28</v>
       </c>
-      <c r="J10" s="726">
+      <c r="J10" s="726" t="n">
         <v>2107.91</v>
       </c>
-      <c r="K10" s="726">
+      <c r="K10" s="726" t="n">
         <v>2269.56</v>
       </c>
-      <c r="L10" s="726">
+      <c r="L10" s="726" t="n">
         <v>2447.03</v>
       </c>
-      <c r="M10" s="726">
+      <c r="M10" s="726" t="n">
         <v>3062.09</v>
       </c>
-      <c r="N10" s="726">
+      <c r="N10" s="726" t="n">
         <v>3395.99</v>
       </c>
-      <c r="O10" s="726">
+      <c r="O10" s="726" t="n">
         <v>3547.57</v>
       </c>
-      <c r="P10" s="726">
+      <c r="P10" s="726" t="n">
         <v>2392.8</v>
       </c>
-      <c r="Q10" s="726">
+      <c r="Q10" s="726" t="n">
         <v>1496.46</v>
       </c>
-      <c r="R10" s="726">
+      <c r="R10" s="726" t="n">
         <v>849.51</v>
       </c>
-      <c r="S10" s="726">
+      <c r="S10" s="726" t="n">
         <v>453.31</v>
       </c>
       <c r="T10" s="149" t="inlineStr">
@@ -6670,52 +6670,52 @@
           <t>T₁ Legacy (Базовый вариант) loan balance</t>
         </is>
       </c>
-      <c r="D13" s="729">
+      <c r="D13" s="729" t="n">
         <v>247.91</v>
       </c>
-      <c r="E13" s="729">
+      <c r="E13" s="729" t="n">
         <v>246.94</v>
       </c>
-      <c r="F13" s="729">
+      <c r="F13" s="729" t="n">
         <v>247.09</v>
       </c>
-      <c r="G13" s="729">
+      <c r="G13" s="729" t="n">
         <v>596.87</v>
       </c>
-      <c r="H13" s="729">
+      <c r="H13" s="729" t="n">
         <v>599.61</v>
       </c>
-      <c r="I13" s="729">
+      <c r="I13" s="729" t="n">
         <v>603.77</v>
       </c>
-      <c r="J13" s="729">
+      <c r="J13" s="729" t="n">
         <v>958.08</v>
       </c>
-      <c r="K13" s="729">
+      <c r="K13" s="729" t="n">
         <v>960.51</v>
       </c>
-      <c r="L13" s="729">
+      <c r="L13" s="729" t="n">
         <v>961.14</v>
       </c>
-      <c r="M13" s="729">
+      <c r="M13" s="729" t="n">
         <v>1261.06</v>
       </c>
-      <c r="N13" s="729">
+      <c r="N13" s="729" t="n">
         <v>1260.48</v>
       </c>
-      <c r="O13" s="729">
+      <c r="O13" s="729" t="n">
         <v>1258.42</v>
       </c>
-      <c r="P13" s="729">
+      <c r="P13" s="729" t="n">
         <v>495.96</v>
       </c>
-      <c r="Q13" s="729">
-        <v>-94.43</v>
-      </c>
-      <c r="R13" s="729">
+      <c r="Q13" s="729" t="n">
+        <v>-94.43000000000001</v>
+      </c>
+      <c r="R13" s="729" t="n">
         <v>-521.79</v>
       </c>
-      <c r="S13" s="729">
+      <c r="S13" s="729" t="n">
         <v>-786.27</v>
       </c>
       <c r="T13" s="514" t="inlineStr">
@@ -6865,52 +6865,52 @@
           <t>TOTAL (ИТОГО) LIABILITIES (ИТОГО ОБЯЗАТЕЛЬСТВА) + EQUITY (ИТОГО ОБЯЗАТЕЛЬСТВА + КАПИТАЛ)</t>
         </is>
       </c>
-      <c r="D16" s="726">
+      <c r="D16" s="726" t="n">
         <v>424.03</v>
       </c>
-      <c r="E16" s="726">
+      <c r="E16" s="726" t="n">
         <v>399.18</v>
       </c>
-      <c r="F16" s="726">
+      <c r="F16" s="726" t="n">
         <v>374.95</v>
       </c>
-      <c r="G16" s="726">
+      <c r="G16" s="726" t="n">
         <v>987.14</v>
       </c>
-      <c r="H16" s="726">
+      <c r="H16" s="726" t="n">
         <v>1076.76</v>
       </c>
-      <c r="I16" s="726">
+      <c r="I16" s="726" t="n">
         <v>1359.28</v>
       </c>
-      <c r="J16" s="726">
+      <c r="J16" s="726" t="n">
         <v>2107.91</v>
       </c>
-      <c r="K16" s="726">
+      <c r="K16" s="726" t="n">
         <v>2269.56</v>
       </c>
-      <c r="L16" s="726">
+      <c r="L16" s="726" t="n">
         <v>2447.03</v>
       </c>
-      <c r="M16" s="726">
+      <c r="M16" s="726" t="n">
         <v>3062.09</v>
       </c>
-      <c r="N16" s="726">
+      <c r="N16" s="726" t="n">
         <v>3395.99</v>
       </c>
-      <c r="O16" s="726">
+      <c r="O16" s="726" t="n">
         <v>3547.57</v>
       </c>
-      <c r="P16" s="726">
+      <c r="P16" s="726" t="n">
         <v>2392.8</v>
       </c>
-      <c r="Q16" s="726">
+      <c r="Q16" s="726" t="n">
         <v>1496.46</v>
       </c>
-      <c r="R16" s="726">
+      <c r="R16" s="726" t="n">
         <v>849.51</v>
       </c>
-      <c r="S16" s="726">
+      <c r="S16" s="726" t="n">
         <v>453.31</v>
       </c>
       <c r="T16" s="149" t="inlineStr">
@@ -6955,53 +6955,53 @@
           <t>Контроль баланса = Активы − (О+К)</t>
         </is>
       </c>
-      <c r="D19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="E19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="F19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="G19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="H19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="I19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="J19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="K19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="L19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="M19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="N19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="O19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="P19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="Q19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="R19" s="731">
-        <v>0.0</v>
-      </c>
-      <c r="S19" s="731">
-        <v>0.0</v>
+      <c r="D19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="731" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="731" t="n">
+        <v>0</v>
       </c>
       <c r="T19" s="164" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
     <row r="31" ht="22" customHeight="1" s="468">
       <c r="B31" s="533" t="inlineStr">
         <is>
-          <t>=</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C31" s="529" t="inlineStr">
@@ -19660,7 +19660,7 @@
     <row r="46">
       <c r="B46" s="556" t="inlineStr">
         <is>
-          <t>Scenario (Сценарий) Base (Базовый) (internal)</t>
+          <t>Scenario (Сценарий) Base (Базовый)</t>
         </is>
       </c>
       <c r="C46" s="473" t="n"/>
@@ -20894,7 +20894,7 @@
     <row r="49" ht="409.6" customHeight="1" s="468">
       <c r="B49" s="436" t="inlineStr">
         <is>
-          <t>V.3  Base (Базовый) scenario IRR (внутренняя норма доходности) = 20.09% превышает hurdle (порог) на +2.09pp. Margin (Маржа) к hurdle (порог) под W₃ (2.09pp) ниже, чем под Internal (Внутренний) W₅ V-D (6.75pp) — это конструктивная особенность W₃ (меньше tiers = меньше upside capture).</t>
+          <t>V.3  Base (Базовый) scenario IRR (внутренняя норма доходности) = 20.09% превышает hurdle (порог) на +2.09pp. Margin (Маржа) к hurdle (порог) под W₃ составляет +2.09pp.</t>
         </is>
       </c>
     </row>
@@ -27770,7 +27770,7 @@
       </c>
       <c r="C30" s="492" t="inlineStr">
         <is>
-          <t>Public export + Internal (Внутренний) с 4 сервисными</t>
+          <t>Public export с 4 сервисными</t>
         </is>
       </c>
       <c r="D30" s="487" t="n"/>
@@ -27808,7 +27808,7 @@
       </c>
       <c r="C32" s="492" t="inlineStr">
         <is>
-          <t>Финализация + computer:// ссылки</t>
+          <t>Финализация + навигационные ссылки</t>
         </is>
       </c>
       <c r="D32" s="487" t="n"/>
@@ -30496,7 +30496,7 @@
       </c>
       <c r="E12" s="595" t="inlineStr">
         <is>
-          <t>Газпром-медиа (internal)</t>
+          <t>Газпром-медиа</t>
         </is>
       </c>
       <c r="F12" s="323" t="n">
@@ -30515,7 +30515,7 @@
       </c>
       <c r="J12" s="610" t="inlineStr">
         <is>
-          <t>Internal (Внутренний) consolidation (Внутренняя консолидация)</t>
+          <t>Consolidation (Консолидация)</t>
         </is>
       </c>
       <c r="K12" s="322" t="inlineStr">
@@ -30538,7 +30538,7 @@
       </c>
       <c r="E13" s="595" t="inlineStr">
         <is>
-          <t>Яндекс (internal)</t>
+          <t>Яндекс</t>
         </is>
       </c>
       <c r="F13" s="323" t="n">
@@ -43824,11 +43824,11 @@
     <mergeCell ref="D42:N42"/>
     <mergeCell ref="B44:N44"/>
     <mergeCell ref="D38:N38"/>
-    <mergeCell ref="B19:N19"/>
+    <mergeCell ref="D23:N23"/>
     <mergeCell ref="D89:N89"/>
     <mergeCell ref="D29:N29"/>
     <mergeCell ref="D85:N85"/>
-    <mergeCell ref="D23:N23"/>
+    <mergeCell ref="B19:N19"/>
     <mergeCell ref="B34:N34"/>
     <mergeCell ref="D14:N14"/>
   </mergeCells>
@@ -43888,23 +43888,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="B2:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="2" customWidth="1" min="10" max="10"/>
+    <col width="2" customWidth="1" style="468" min="1" max="1"/>
+    <col width="6" customWidth="1" style="468" min="2" max="2"/>
+    <col width="34" customWidth="1" style="468" min="3" max="3"/>
+    <col width="10" customWidth="1" style="468" min="4" max="4"/>
+    <col width="16" customWidth="1" style="468" min="5" max="5"/>
+    <col width="16" customWidth="1" style="468" min="6" max="6"/>
+    <col width="16" customWidth="1" style="468" min="7" max="7"/>
+    <col width="16" customWidth="1" style="468" min="8" max="8"/>
+    <col width="16" customWidth="1" style="468" min="9" max="9"/>
+    <col width="2" customWidth="1" style="468" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="30" customHeight="1" s="468">
       <c r="B2" s="666" t="inlineStr">
         <is>
           <t>FOT (фонд оплаты труда) / Штат — Модель A₂ (Market-Based)</t>
@@ -43918,8 +43917,7 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="32" customHeight="1" s="468">
       <c r="B5" s="668" t="inlineStr">
         <is>
           <t>#</t>
@@ -43961,7 +43959,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
+    <row r="6" ht="20" customHeight="1" s="468">
       <c r="B6" s="669" t="n">
         <v>1</v>
       </c>
@@ -43993,7 +43991,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
+    <row r="7" ht="20" customHeight="1" s="468">
       <c r="B7" s="669" t="n">
         <v>2</v>
       </c>
@@ -44025,7 +44023,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
+    <row r="8" ht="20" customHeight="1" s="468">
       <c r="B8" s="669" t="n">
         <v>3</v>
       </c>
@@ -44057,7 +44055,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
+    <row r="9" ht="20" customHeight="1" s="468">
       <c r="B9" s="669" t="n">
         <v>4</v>
       </c>
@@ -44089,7 +44087,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="10" ht="20" customHeight="1" s="468">
       <c r="B10" s="669" t="n">
         <v>5</v>
       </c>
@@ -44121,7 +44119,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11" ht="20" customHeight="1" s="468">
       <c r="B11" s="669" t="n">
         <v>6</v>
       </c>
@@ -44153,7 +44151,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
+    <row r="12" ht="20" customHeight="1" s="468">
       <c r="B12" s="669" t="n">
         <v>7</v>
       </c>
@@ -44185,7 +44183,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
+    <row r="13" ht="20" customHeight="1" s="468">
       <c r="B13" s="669" t="n">
         <v>8</v>
       </c>
@@ -44217,7 +44215,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="26" customHeight="1">
+    <row r="14" ht="26" customHeight="1" s="468">
       <c r="B14" s="675" t="n"/>
       <c r="C14" s="676" t="inlineStr">
         <is>
@@ -44241,15 +44239,14 @@
         <v>100152000</v>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16" ht="20" customHeight="1">
+    <row r="16" ht="20" customHeight="1" s="468">
       <c r="B16" s="679" t="inlineStr">
         <is>
           <t>ФОТ A₂ за 3 года (2026–2028), млн ₽</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="28" customHeight="1" s="468">
       <c r="C17" s="668" t="inlineStr">
         <is>
           <t>Год</t>
@@ -44286,7 +44283,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18" ht="20" customHeight="1" s="468">
       <c r="C18" s="680" t="n">
         <v>2026</v>
       </c>
@@ -44311,7 +44308,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
+    <row r="19" ht="20" customHeight="1" s="468">
       <c r="C19" s="680" t="n">
         <v>2027</v>
       </c>
@@ -44340,7 +44337,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
+    <row r="20" ht="20" customHeight="1" s="468">
       <c r="C20" s="680" t="n">
         <v>2028</v>
       </c>
@@ -44369,7 +44366,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
+    <row r="21" ht="24" customHeight="1" s="468">
       <c r="C21" s="686" t="inlineStr">
         <is>
           <t>Σ 2026–2028</t>
@@ -44398,8 +44395,7 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23" ht="32" customHeight="1">
+    <row r="23" ht="32" customHeight="1" s="468">
       <c r="B23" s="688" t="inlineStr">
         <is>
           <t>⚫ Модель A₂ «Market-Based»: 43 чел, оклады по P50 рынка МСК 2025-2026. Индексация 8%/год. Σ ФОТ 2026-2028 ≈ 325 млн ₽. Источники: hh.ru, ГородРабот, DreamJob.</t>
@@ -47953,24 +47949,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="B2:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="2" customWidth="1" min="11" max="11"/>
+    <col width="2" customWidth="1" style="468" min="1" max="1"/>
+    <col width="32" customWidth="1" style="468" min="2" max="2"/>
+    <col width="12" customWidth="1" style="468" min="3" max="3"/>
+    <col width="12" customWidth="1" style="468" min="4" max="4"/>
+    <col width="12" customWidth="1" style="468" min="5" max="5"/>
+    <col width="12" customWidth="1" style="468" min="6" max="6"/>
+    <col width="12" customWidth="1" style="468" min="7" max="7"/>
+    <col width="12" customWidth="1" style="468" min="8" max="8"/>
+    <col width="12" customWidth="1" style="468" min="9" max="9"/>
+    <col width="12" customWidth="1" style="468" min="10" max="10"/>
+    <col width="2" customWidth="1" style="468" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="30" customHeight="1" s="468">
       <c r="B2" s="666" t="inlineStr">
         <is>
           <t>FOT (фонд оплаты труда) / Штат — Модель A₂ Dynamic (Динамический) (Market + 8% индексация)</t>
@@ -47984,15 +47979,14 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5" ht="20" customHeight="1">
+    <row r="5" ht="20" customHeight="1" s="468">
       <c r="B5" s="679" t="inlineStr">
         <is>
           <t>ПАРАМЕТРЫ ДИНАМИКИ (ввод)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="22" customHeight="1" s="468">
       <c r="B6" s="668" t="inlineStr">
         <is>
           <t>Параметр</t>
@@ -48034,7 +48028,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
+    <row r="7" ht="20" customHeight="1" s="468">
       <c r="B7" s="689" t="inlineStr">
         <is>
           <t>Штат (чел.)</t>
@@ -48062,7 +48056,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8" ht="18" customHeight="1" s="468">
       <c r="B8" s="670" t="inlineStr">
         <is>
           <t>Индекс оклада (база 2026=1.00)</t>
@@ -48090,7 +48084,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
+    <row r="9" ht="18" customHeight="1" s="468">
       <c r="B9" s="670" t="inlineStr">
         <is>
           <t>Ср. оклад gross (₽/мес, база 2026)</t>
@@ -48118,7 +48112,7 @@
         <v>237390.6976744186</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="18" customHeight="1" s="468">
       <c r="B10" s="670" t="inlineStr">
         <is>
           <t>ФОТ gross / мес</t>
@@ -48153,7 +48147,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11" ht="20" customHeight="1" s="468">
       <c r="B11" s="689" t="inlineStr">
         <is>
           <t>ФОТ с налогами / мес (×1.30)</t>
@@ -48188,7 +48182,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
+    <row r="12" ht="24" customHeight="1" s="468">
       <c r="B12" s="676" t="inlineStr">
         <is>
           <t>ФОТ годовой (млн ₽)</t>
@@ -48223,15 +48217,14 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14" ht="20" customHeight="1">
+    <row r="14" ht="20" customHeight="1" s="468">
       <c r="B14" s="679" t="inlineStr">
         <is>
           <t>ПОКВАРТАЛЬНАЯ РАЗБИВКА 2026–2028 (млн ₽)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="22" customHeight="1" s="468">
       <c r="B15" s="668" t="inlineStr">
         <is>
           <t>Квартал</t>
@@ -48263,7 +48256,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
+    <row r="16" ht="20" customHeight="1" s="468">
       <c r="B16" s="691" t="inlineStr">
         <is>
           <t>2026</t>
@@ -48290,7 +48283,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
+    <row r="17" ht="20" customHeight="1" s="468">
       <c r="B17" s="691" t="inlineStr">
         <is>
           <t>2027</t>
@@ -48317,7 +48310,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18" ht="20" customHeight="1" s="468">
       <c r="B18" s="691" t="inlineStr">
         <is>
           <t>2028</t>
@@ -48344,7 +48337,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
+    <row r="19" ht="24" customHeight="1" s="468">
       <c r="B19" s="686" t="inlineStr">
         <is>
           <t>Σ 2026–2028</t>
@@ -48371,15 +48364,14 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21" ht="20" customHeight="1">
+    <row r="21" ht="20" customHeight="1" s="468">
       <c r="B21" s="679" t="inlineStr">
         <is>
           <t>СРАВНЕНИЕ A₁ Fixed (Фиксированный) vs A₂ Dynamic (Динамический)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
+    <row r="22" ht="22" customHeight="1" s="468">
       <c r="B22" s="668" t="inlineStr">
         <is>
           <t>Период</t>
@@ -48406,7 +48398,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
+    <row r="23" ht="20" customHeight="1" s="468">
       <c r="B23" s="695" t="n">
         <v>2026</v>
       </c>
@@ -48426,7 +48418,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24" ht="20" customHeight="1" s="468">
       <c r="B24" s="695" t="n">
         <v>2027</v>
       </c>
@@ -48446,7 +48438,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
+    <row r="25" ht="20" customHeight="1" s="468">
       <c r="B25" s="695" t="n">
         <v>2028</v>
       </c>
@@ -48466,7 +48458,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
+    <row r="26" ht="24" customHeight="1" s="468">
       <c r="B26" s="686" t="inlineStr">
         <is>
           <t>Σ 3 года</t>
@@ -48489,8 +48481,7 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28" ht="50" customHeight="1">
+    <row r="28" ht="50" customHeight="1" s="468">
       <c r="B28" s="688" t="inlineStr">
         <is>
           <t>⚫ Модель A₂ «Full Dynamic (Динамический)»: штат растёт 50→60→70 (pre-IPO (первичное размещение) команда), оклады индексируются 7%/год (CPI 6.5% + премия). Для 2026–2028 разница с A₁ отражает реалистичный рост OPEX (Операционные расходы) и используется в pessimistic scenarios. Для верификации якоря EBITDA (прибыль до вычетов) = 3 000 млн ₽ используется A₁. В дальнейшем можно переключить P&amp;L через selector на A₂.</t>

</xml_diff>